<commit_message>
Refactor spell casting mechanics and enhance user interaction
- Improved spell selection logic to allow users to cancel casting spells.
- Updated UI elements to better indicate spell selection status and enhance user feedback.
- Enhanced tests to validate the integration of spell cancellation features within the combat system.
</commit_message>
<xml_diff>
--- a/spell_types.xlsx
+++ b/spell_types.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_0E0D2663A25BDFAF6A16D8E49D42A91495351BD0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{966B8B31-BF7C-48F8-AB89-A73313037E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3810" yWindow="4260" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Spells" sheetId="1" r:id="rId1"/>

</xml_diff>